<commit_message>
draw the null band as a quantile so the figure stops contradicting its own p-value
</commit_message>
<xml_diff>
--- a/04_Features/modules/loso_refit/c_data/loso_refit.xlsx
+++ b/04_Features/modules/loso_refit/c_data/loso_refit.xlsx
@@ -8,12 +8,13 @@
   <sheets>
     <sheet name="refit_summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="module_stability" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="provenance" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t xml:space="preserve">stage</t>
   </si>
@@ -57,33 +58,45 @@
     <t xml:space="preserve">modules</t>
   </si>
   <si>
+    <t xml:space="preserve">acute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_mcsa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lasso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ridge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">svm</t>
+  </si>
+  <si>
     <t xml:space="preserve">T2</t>
   </si>
   <si>
-    <t xml:space="preserve">d_mcsa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">enet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lasso</t>
-  </si>
-  <si>
     <t xml:space="preserve">T3</t>
   </si>
   <si>
+    <t xml:space="preserve">plain</t>
+  </si>
+  <si>
     <t xml:space="preserve">rf</t>
   </si>
   <si>
     <t xml:space="preserve">total</t>
   </si>
   <si>
+    <t xml:space="preserve">trajectory</t>
+  </si>
+  <si>
     <t xml:space="preserve">spls</t>
   </si>
   <si>
-    <t xml:space="preserve">trajectory</t>
-  </si>
-  <si>
     <t xml:space="preserve">module</t>
   </si>
   <si>
@@ -126,10 +139,19 @@
     <t xml:space="preserve">red</t>
   </si>
   <si>
+    <t xml:space="preserve">tan</t>
+  </si>
+  <si>
     <t xml:space="preserve">turquoise</t>
   </si>
   <si>
     <t xml:space="preserve">yellow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fingerprint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21f8a1d53f92</t>
   </si>
 </sst>
 </file>
@@ -513,7 +535,7 @@
         <v>16</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2160515511346</v>
+        <v>0.444504844977317</v>
       </c>
       <c r="G2" t="n">
         <v>-0.14795918367347</v>
@@ -522,13 +544,13 @@
         <v>-0.14795918367347</v>
       </c>
       <c r="I2" t="n">
-        <v>0.82089552238806</v>
+        <v>0.81592039800995</v>
       </c>
       <c r="J2" t="n">
-        <v>0.36401073480807</v>
+        <v>0.592464028650787</v>
       </c>
       <c r="K2" t="n">
-        <v>0.36401073480807</v>
+        <v>0.592464028650787</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -551,7 +573,7 @@
         <v>17</v>
       </c>
       <c r="F3" t="n">
-        <v>0.249732775292857</v>
+        <v>0.462372213177816</v>
       </c>
       <c r="G3" t="n">
         <v>-0.14795918367347</v>
@@ -560,13 +582,13 @@
         <v>-0.14795918367347</v>
       </c>
       <c r="I3" t="n">
-        <v>0.81592039800995</v>
+        <v>0.810945273631841</v>
       </c>
       <c r="J3" t="n">
-        <v>0.397691958966326</v>
+        <v>0.610331396851286</v>
       </c>
       <c r="K3" t="n">
-        <v>0.397691958966326</v>
+        <v>0.610331396851286</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -580,34 +602,34 @@
         <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
         <v>15</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F4" t="n">
-        <v>0.309257343662561</v>
+        <v>0.395420724337231</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.0779980153842508</v>
+        <v>-0.14795918367347</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.207549805410135</v>
+        <v>-0.14795918367347</v>
       </c>
       <c r="I4" t="n">
-        <v>0.338308457711443</v>
+        <v>0.810945273631841</v>
       </c>
       <c r="J4" t="n">
-        <v>0.516807149072696</v>
+        <v>0.5433799080107</v>
       </c>
       <c r="K4" t="n">
-        <v>0.387255359046812</v>
+        <v>0.5433799080107</v>
       </c>
       <c r="L4" t="n">
-        <v>0.129551790025884</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -618,34 +640,34 @@
         <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D5" t="s">
         <v>15</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F5" t="n">
-        <v>0.214388914026353</v>
+        <v>0.381321799187095</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.313415932943927</v>
+        <v>-0.4556329596711</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.301514641086706</v>
+        <v>-0.428200529604371</v>
       </c>
       <c r="I5" t="n">
-        <v>0.338308457711443</v>
+        <v>0.492537313432836</v>
       </c>
       <c r="J5" t="n">
-        <v>0.515903555113059</v>
+        <v>0.809522328791466</v>
       </c>
       <c r="K5" t="n">
-        <v>0.52780484697028</v>
+        <v>0.836954758858194</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.0119012918572212</v>
+        <v>-0.0274324300667288</v>
       </c>
     </row>
     <row r="6">
@@ -656,7 +678,7 @@
         <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D6" t="s">
         <v>15</v>
@@ -665,22 +687,22 @@
         <v>16</v>
       </c>
       <c r="F6" t="n">
-        <v>0.282583392968293</v>
+        <v>0.0701252400887916</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.159763313609467</v>
+        <v>-0.14795918367347</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.159763313609467</v>
+        <v>-0.14795918367347</v>
       </c>
       <c r="I6" t="n">
-        <v>0.378109452736318</v>
+        <v>0.805970149253731</v>
       </c>
       <c r="J6" t="n">
-        <v>0.44234670657776</v>
+        <v>0.218084423762261</v>
       </c>
       <c r="K6" t="n">
-        <v>0.44234670657776</v>
+        <v>0.218084423762261</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
@@ -694,7 +716,7 @@
         <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
         <v>15</v>
@@ -703,22 +725,22 @@
         <v>17</v>
       </c>
       <c r="F7" t="n">
-        <v>0.262322625063435</v>
+        <v>0.177100266471497</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.159763313609467</v>
+        <v>-0.14795918367347</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.159763313609467</v>
+        <v>-0.14795918367347</v>
       </c>
       <c r="I7" t="n">
-        <v>0.398009950248756</v>
+        <v>0.800995024875622</v>
       </c>
       <c r="J7" t="n">
-        <v>0.422085938672902</v>
+        <v>0.325059450144967</v>
       </c>
       <c r="K7" t="n">
-        <v>0.422085938672902</v>
+        <v>0.325059450144967</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -732,34 +754,34 @@
         <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D8" t="s">
         <v>15</v>
       </c>
       <c r="E8" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F8" t="n">
-        <v>0.385810185737778</v>
+        <v>0.140992211958394</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.0481455557948103</v>
+        <v>-0.242597386943361</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.0936150131806179</v>
+        <v>-0.210171391206952</v>
       </c>
       <c r="I8" t="n">
-        <v>0.253731343283582</v>
+        <v>0.208955223880597</v>
       </c>
       <c r="J8" t="n">
-        <v>0.479425198918396</v>
+        <v>0.351163603165347</v>
       </c>
       <c r="K8" t="n">
-        <v>0.433955741532588</v>
+        <v>0.383589598901755</v>
       </c>
       <c r="L8" t="n">
-        <v>0.0454694573858077</v>
+        <v>-0.0324259957364086</v>
       </c>
     </row>
     <row r="9">
@@ -770,34 +792,224 @@
         <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D9" t="s">
         <v>15</v>
       </c>
       <c r="E9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F9" t="n">
-        <v>0.36795135249738</v>
+        <v>0.249482477508396</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.244478204343245</v>
+        <v>-0.392547898540062</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.211204123504218</v>
+        <v>-0.341990759105408</v>
       </c>
       <c r="I9" t="n">
-        <v>0.223880597014925</v>
+        <v>0.557213930348259</v>
       </c>
       <c r="J9" t="n">
-        <v>0.579155476001598</v>
+        <v>0.591473236613804</v>
       </c>
       <c r="K9" t="n">
-        <v>0.612429556840625</v>
+        <v>0.642030376048458</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.0332740808390271</v>
+        <v>-0.0505571394346542</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.392983399454889</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-0.76096669608306</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-0.695800208523955</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.72636815920398</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1.08878360797884</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1.15395009553795</v>
+      </c>
+      <c r="L10" t="n">
+        <v>-0.0651664875591054</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.417565383061029</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-0.159763313609467</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-0.159763313609467</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.398009950248756</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.577328696670496</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.577328696670496</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.150863640518479</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-0.159763313609467</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-0.159763313609467</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.407960199004975</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.310626954127946</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.310626954127946</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.37156217891133</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-0.189311360728277</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-0.136716913530948</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.298507462686567</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.508279092442278</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.560873539639607</v>
+      </c>
+      <c r="L13" t="n">
+        <v>-0.0525944471973285</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.400204457349602</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-0.28033637890863</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-0.222073239668982</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.228855721393035</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.622277697018584</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.680540836258232</v>
+      </c>
+      <c r="L14" t="n">
+        <v>-0.0582631392396487</v>
       </c>
     </row>
   </sheetData>
@@ -813,149 +1025,149 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B2" t="n">
-        <v>0.392848713237482</v>
+        <v>0.491207288829881</v>
       </c>
       <c r="C2" t="n">
-        <v>0.208333333333333</v>
+        <v>0.303703703703704</v>
       </c>
       <c r="D2" t="n">
         <v>16</v>
       </c>
       <c r="E2" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B3" t="n">
-        <v>0.533381687884177</v>
+        <v>0.638793240829182</v>
       </c>
       <c r="C3" t="n">
-        <v>0.390350877192982</v>
+        <v>0.455172413793103</v>
       </c>
       <c r="D3" t="n">
         <v>16</v>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B4" t="n">
-        <v>0.456717814398046</v>
+        <v>0.550345661474563</v>
       </c>
       <c r="C4" t="n">
-        <v>0.267857142857143</v>
+        <v>0.399267399267399</v>
       </c>
       <c r="D4" t="n">
         <v>16</v>
       </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B5" t="n">
-        <v>0.616283434304412</v>
+        <v>0.364550064733596</v>
       </c>
       <c r="C5" t="n">
-        <v>0.44578313253012</v>
+        <v>0.190283400809717</v>
       </c>
       <c r="D5" t="n">
         <v>16</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B6" t="n">
-        <v>0.536991779737618</v>
+        <v>0.384378327283981</v>
       </c>
       <c r="C6" t="n">
-        <v>0.207070707070707</v>
+        <v>0.117424242424242</v>
       </c>
       <c r="D6" t="n">
         <v>16</v>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B7" t="n">
-        <v>0.853836519990896</v>
+        <v>0.512358541458329</v>
       </c>
       <c r="C7" t="n">
-        <v>0.666666666666667</v>
+        <v>0.149253731343284</v>
       </c>
       <c r="D7" t="n">
         <v>16</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B8" t="n">
-        <v>0.462187563531427</v>
+        <v>0.837031261065614</v>
       </c>
       <c r="C8" t="n">
-        <v>0.115131578947368</v>
+        <v>0.616822429906542</v>
       </c>
       <c r="D8" t="n">
         <v>16</v>
       </c>
       <c r="E8" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B9" t="n">
-        <v>0.376967366269988</v>
+        <v>0.357028385028763</v>
       </c>
       <c r="C9" t="n">
-        <v>0.25</v>
+        <v>0.215859030837004</v>
       </c>
       <c r="D9" t="n">
         <v>16</v>
@@ -966,53 +1178,91 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B10" t="n">
-        <v>0.497336879208876</v>
+        <v>0.652067545553724</v>
       </c>
       <c r="C10" t="n">
-        <v>0.213235294117647</v>
+        <v>0.303333333333333</v>
       </c>
       <c r="D10" t="n">
         <v>16</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B11" t="n">
-        <v>0.882277104195404</v>
+        <v>0.485896637069934</v>
       </c>
       <c r="C11" t="n">
-        <v>0.796650717703349</v>
+        <v>0.115555555555556</v>
       </c>
       <c r="D11" t="n">
         <v>16</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B12" t="n">
-        <v>0.609363488973251</v>
+        <v>0.886888258888022</v>
       </c>
       <c r="C12" t="n">
-        <v>0.376237623762376</v>
+        <v>0.782178217821782</v>
       </c>
       <c r="D12" t="n">
         <v>16</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.490317823558289</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.288770053475936</v>
+      </c>
+      <c r="D13" t="n">
+        <v>16</v>
+      </c>
+      <c r="E13" t="n">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>